<commit_message>
added the sdtmct version to library tab
</commit_message>
<xml_diff>
--- a/rules/CORE-002117/positive/01/data/CORE-002117-positive-01.xlsx
+++ b/rules/CORE-002117/positive/01/data/CORE-002117-positive-01.xlsx
@@ -467,7 +467,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B3"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="str">
@@ -478,16 +478,24 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="str">
+      <c r="A2" s="2" t="str">
         <v>sdtmig</v>
       </c>
-      <c r="B2" s="3" t="str">
+      <c r="B2" s="2" t="str">
         <v>3-4</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="str">
+        <v>sdtmct</v>
+      </c>
+      <c r="B3" s="3" t="str">
+        <v>204-09-27</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B3"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>